<commit_message>
Liu retest the updated codes with minor modifications; a new plot script is added to work with C0003R02
</commit_message>
<xml_diff>
--- a/data/C0004/C0004R01_PARK25_AC_1D_SCAN.xlsx
+++ b/data/C0004/C0004R01_PARK25_AC_1D_SCAN.xlsx
@@ -455,7 +455,7 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="19" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
@@ -587,10 +587,10 @@
         <v>19</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.002396728974089701</v>
+        <v>0.02593481266904006</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>3.307485984243787</v>
+        <v>35.79004148327528</v>
       </c>
       <c r="H2" s="4" t="n">
         <v>45.35221322014578</v>
@@ -648,10 +648,10 @@
         <v>20</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>0.002641479713652297</v>
+        <v>0.02723849278577916</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>3.645242004840171</v>
+        <v>37.58912004437524</v>
       </c>
       <c r="H3" s="4" t="n">
         <v>45.22349700005135</v>
@@ -709,10 +709,10 @@
         <v>21</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.002898126754191331</v>
+        <v>0.02854959673718338</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>3.999414920784037</v>
+        <v>39.39844349731307</v>
       </c>
       <c r="H4" s="4" t="n">
         <v>45.10485715458326</v>
@@ -770,10 +770,10 @@
         <v>22</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.003166670095706803</v>
+        <v>0.02986900617507107</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4.370004732075388</v>
+        <v>41.21922852159808</v>
       </c>
       <c r="H5" s="4" t="n">
         <v>44.995176019449</v>
@@ -831,10 +831,10 @@
         <v>23</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.003447109738198712</v>
+        <v>0.03119758720222467</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4.757011438714222</v>
+        <v>43.05267033907005</v>
       </c>
       <c r="H6" s="4" t="n">
         <v>44.89349206415539</v>
@@ -892,10 +892,10 @@
         <v>19</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>0.002428641212177403</v>
+        <v>0.02628013244678785</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>3.351524872804816</v>
+        <v>36.26658277656724</v>
       </c>
       <c r="H7" s="4" t="n">
         <v>50.40776704005317</v>
@@ -953,10 +953,10 @@
         <v>20</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.002676650786575936</v>
+        <v>0.02760117095103149</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>3.693778085474792</v>
+        <v>38.08961591242345</v>
       </c>
       <c r="H8" s="4" t="n">
         <v>50.27786741215457</v>
@@ -1014,10 +1014,10 @@
         <v>21</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0.002936715060164984</v>
+        <v>0.02892973213765391</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>4.052666783027679</v>
+        <v>39.92303034996239</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>50.15810314910172</v>
@@ -1075,10 +1075,10 @@
         <v>22</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>0.003208834032944548</v>
+        <v>0.03026670939759081</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>4.428190965463475</v>
+        <v>41.76805896867532</v>
       </c>
       <c r="H10" s="4" t="n">
         <v>50.04735435433316</v>
@@ -1136,10 +1136,10 @@
         <v>23</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.003493007704914626</v>
+        <v>0.03161298036570799</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>4.820350632782183</v>
+        <v>43.62591290467703</v>
       </c>
       <c r="H11" s="4" t="n">
         <v>49.94465686615955</v>
@@ -1197,10 +1197,10 @@
         <v>19</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.002460329809319224</v>
+        <v>0.02662303222373487</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>3.39525513686053</v>
+        <v>36.73978446875412</v>
       </c>
       <c r="H12" s="4" t="n">
         <v>55.46262295036126</v>
@@ -1258,10 +1258,10 @@
         <v>20</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.002711575380641067</v>
+        <v>0.02796130746791354</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>3.741974025284673</v>
+        <v>38.58660430572068</v>
       </c>
       <c r="H13" s="4" t="n">
         <v>55.3315670127763</v>
@@ -1319,10 +1319,10 @@
         <v>21</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>0.002975032939312911</v>
+        <v>0.02930720354945993</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>4.105545456251817</v>
+        <v>40.44394089825471</v>
       </c>
       <c r="H14" s="4" t="n">
         <v>55.21070273458488</v>
@@ -1380,10 +1380,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0.003250702485334755</v>
+        <v>0.03066162551615941</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>4.485969429761962</v>
+        <v>42.31304321229998</v>
       </c>
       <c r="H15" s="4" t="n">
         <v>55.098908342869</v>
@@ -1441,10 +1441,10 @@
         <v>23</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>0.003538584018706599</v>
+        <v>0.03202546245414421</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>4.883245945815107</v>
+        <v>44.19513818671901</v>
       </c>
       <c r="H16" s="4" t="n">
         <v>54.99521734423036</v>
@@ -1502,10 +1502,10 @@
         <v>19</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>0.002491798875350332</v>
+        <v>0.02696355647207897</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>3.438682447983458</v>
+        <v>37.20970793146897</v>
       </c>
       <c r="H17" s="4" t="n">
         <v>60.51679029341818</v>
@@ -1563,10 +1563,10 @@
         <v>20</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>0.002746258025373697</v>
+        <v>0.02831894904413268</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>3.789836075015702</v>
+        <v>39.08014968090311</v>
       </c>
       <c r="H18" s="4" t="n">
         <v>60.38460469011161</v>
@@ -1624,10 +1624,10 @@
         <v>21</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>0.00301308536125136</v>
+        <v>0.0296820599285485</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>4.158057798526876</v>
+        <v>40.96124270139693</v>
       </c>
       <c r="H19" s="4" t="n">
         <v>60.26266440703396</v>
@@ -1685,10 +1685,10 @@
         <v>22</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>0.003292280882983317</v>
+        <v>0.03105380574920552</v>
       </c>
       <c r="G20" s="4" t="n">
-        <v>4.543347618516977</v>
+        <v>42.85425193390361</v>
       </c>
       <c r="H20" s="4" t="n">
         <v>60.14984614020961</v>
@@ -1746,10 +1746,10 @@
         <v>23</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>0.003583844590569569</v>
+        <v>0.03243508696417081</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>4.945705534986005</v>
+        <v>44.76042001055571</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>60.04518135555108</v>
@@ -1807,10 +1807,10 @@
         <v>19</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>0.002523052415836009</v>
+        <v>0.02730174853572195</v>
       </c>
       <c r="G22" s="4" t="n">
-        <v>3.481812333853693</v>
+        <v>37.67641297929629</v>
       </c>
       <c r="H22" s="4" t="n">
         <v>65.57027817084963</v>
@@ -1868,10 +1868,10 @@
         <v>20</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>0.002780703135382051</v>
+        <v>0.0286741412023835</v>
       </c>
       <c r="G23" s="4" t="n">
-        <v>3.837370326827231</v>
+        <v>39.57031485928923</v>
       </c>
       <c r="H23" s="4" t="n">
         <v>65.4369890959878</v>
@@ -1929,10 +1929,10 @@
         <v>21</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>0.003050877169513346</v>
+        <v>0.03005434898881416</v>
       </c>
       <c r="G24" s="4" t="n">
-        <v>4.210210493928417</v>
+        <v>41.47500160456354</v>
       </c>
       <c r="H24" s="4" t="n">
         <v>65.31399642962884</v>
@@ -1990,10 +1990,10 @@
         <v>22</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>0.003333574518229891</v>
+        <v>0.03144330001570434</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>4.60033283515725</v>
+        <v>43.39175402167199</v>
       </c>
       <c r="H25" s="4" t="n">
         <v>65.20017567160524</v>
@@ -2051,10 +2051,10 @@
         <v>23</v>
       </c>
       <c r="F26" s="4" t="n">
-        <v>0.003628795181531689</v>
+        <v>0.03284190603517174</v>
       </c>
       <c r="G26" s="4" t="n">
-        <v>5.007737350513731</v>
+        <v>45.321830328537</v>
       </c>
       <c r="H26" s="4" t="n">
         <v>65.09455652982655</v>
@@ -2112,10 +2112,10 @@
         <v>19</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>0.01013408801947973</v>
+        <v>0.1037392506761602</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>13.98504146688203</v>
+        <v>143.1601659331011</v>
       </c>
       <c r="H27" s="4" t="n">
         <v>42.74357574045806</v>
@@ -2173,10 +2173,10 @@
         <v>20</v>
       </c>
       <c r="F28" s="4" t="n">
-        <v>0.01116896745907184</v>
+        <v>0.1089539711431167</v>
       </c>
       <c r="G28" s="4" t="n">
-        <v>15.41317509351914</v>
+        <v>150.356480177501</v>
       </c>
       <c r="H28" s="4" t="n">
         <v>42.6562012927463</v>
@@ -2234,10 +2234,10 @@
         <v>21</v>
       </c>
       <c r="F29" s="4" t="n">
-        <v>0.01225414802261444</v>
+        <v>0.1141983869487335</v>
       </c>
       <c r="G29" s="4" t="n">
-        <v>16.91072427120793</v>
+        <v>157.5937739892523</v>
       </c>
       <c r="H29" s="4" t="n">
         <v>42.57644109923064</v>
@@ -2295,10 +2295,10 @@
         <v>22</v>
       </c>
       <c r="F30" s="4" t="n">
-        <v>0.01338962971010755</v>
+        <v>0.1194760247002843</v>
       </c>
       <c r="G30" s="4" t="n">
-        <v>18.47768899994842</v>
+        <v>164.8769140863923</v>
       </c>
       <c r="H30" s="4" t="n">
         <v>42.50334781382457</v>
@@ -2356,10 +2356,10 @@
         <v>23</v>
       </c>
       <c r="F31" s="4" t="n">
-        <v>0.01457541252155116</v>
+        <v>0.1247903488088987</v>
       </c>
       <c r="G31" s="4" t="n">
-        <v>20.1140692797406</v>
+        <v>172.2106813562802</v>
       </c>
       <c r="H31" s="4" t="n">
         <v>42.43612402365883</v>
@@ -2417,10 +2417,10 @@
         <v>19</v>
       </c>
       <c r="F32" s="4" t="n">
-        <v>0.009788878218848197</v>
+        <v>0.1051205297871514</v>
       </c>
       <c r="G32" s="4" t="n">
-        <v>13.50865194201051</v>
+        <v>145.066331106269</v>
       </c>
       <c r="H32" s="4" t="n">
         <v>47.78628458061043</v>
@@ -2478,10 +2478,10 @@
         <v>20</v>
       </c>
       <c r="F33" s="4" t="n">
-        <v>0.0107885052978596</v>
+        <v>0.110404683804126</v>
       </c>
       <c r="G33" s="4" t="n">
-        <v>14.88813731104625</v>
+        <v>152.3584636496938</v>
       </c>
       <c r="H33" s="4" t="n">
         <v>47.69764927452142</v>
@@ -2539,10 +2539,10 @@
         <v>21</v>
       </c>
       <c r="F34" s="4" t="n">
-        <v>0.01183672003228471</v>
+        <v>0.1157189285506156</v>
       </c>
       <c r="G34" s="4" t="n">
-        <v>16.3346736445529</v>
+        <v>159.6921213998496</v>
       </c>
       <c r="H34" s="4" t="n">
         <v>47.61672790683462</v>
@@ -2600,10 +2600,10 @@
         <v>22</v>
       </c>
       <c r="F35" s="4" t="n">
-        <v>0.01293352242212352</v>
+        <v>0.1210668375903633</v>
       </c>
       <c r="G35" s="4" t="n">
-        <v>17.84826094253047</v>
+        <v>167.0722358747013</v>
       </c>
       <c r="H35" s="4" t="n">
         <v>47.54256213730193</v>
@@ -2661,10 +2661,10 @@
         <v>23</v>
       </c>
       <c r="F36" s="4" t="n">
-        <v>0.01407891246737604</v>
+        <v>0.126451921462832</v>
       </c>
       <c r="G36" s="4" t="n">
-        <v>19.42889920497894</v>
+        <v>174.5036516187081</v>
       </c>
       <c r="H36" s="4" t="n">
         <v>47.4743450542931</v>
@@ -2722,10 +2722,10 @@
         <v>19</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>0.009841319237276897</v>
+        <v>0.1064921288949395</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>13.58102054744212</v>
+        <v>146.9591378750165</v>
       </c>
       <c r="H37" s="4" t="n">
         <v>52.82867331219183</v>
@@ -2783,10 +2783,10 @@
         <v>20</v>
       </c>
       <c r="F38" s="4" t="n">
-        <v>0.01084630152256427</v>
+        <v>0.1118452298716542</v>
       </c>
       <c r="G38" s="4" t="n">
-        <v>14.96789610113869</v>
+        <v>154.3464172228827</v>
       </c>
       <c r="H38" s="4" t="n">
         <v>52.73878901208428</v>
@@ -2844,10 +2844,10 @@
         <v>21</v>
       </c>
       <c r="F39" s="4" t="n">
-        <v>0.01190013175725164</v>
+        <v>0.1172288141978397</v>
       </c>
       <c r="G39" s="4" t="n">
-        <v>16.42218182500727</v>
+        <v>161.7757635930188</v>
       </c>
       <c r="H39" s="4" t="n">
         <v>52.6567169385884</v>
@@ -2905,10 +2905,10 @@
         <v>22</v>
       </c>
       <c r="F40" s="4" t="n">
-        <v>0.01300280994133902</v>
+        <v>0.1226465020646376</v>
       </c>
       <c r="G40" s="4" t="n">
-        <v>17.94387771904785</v>
+        <v>169.2521728491999</v>
       </c>
       <c r="H40" s="4" t="n">
         <v>52.58148797759323</v>
@@ -2966,10 +2966,10 @@
         <v>23</v>
       </c>
       <c r="F41" s="4" t="n">
-        <v>0.0141543360748264</v>
+        <v>0.1281018498165769</v>
       </c>
       <c r="G41" s="4" t="n">
-        <v>19.53298378326043</v>
+        <v>176.7805527468761</v>
       </c>
       <c r="H41" s="4" t="n">
         <v>52.51228589660823</v>
@@ -3027,10 +3027,10 @@
         <v>19</v>
       </c>
       <c r="F42" s="4" t="n">
-        <v>0.009967195501401328</v>
+        <v>0.1078542258883159</v>
       </c>
       <c r="G42" s="4" t="n">
-        <v>13.75472979193383</v>
+        <v>148.8388317258759</v>
       </c>
       <c r="H42" s="4" t="n">
         <v>57.87074283536434</v>
@@ -3088,10 +3088,10 @@
         <v>20</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0.01098503210149479</v>
+        <v>0.1132757961765307</v>
       </c>
       <c r="G43" s="4" t="n">
-        <v>15.15934430006281</v>
+        <v>156.3205987236124</v>
       </c>
       <c r="H43" s="4" t="n">
         <v>57.77962144118474</v>
@@ -3149,10 +3149,10 @@
         <v>21</v>
       </c>
       <c r="F44" s="4" t="n">
-        <v>0.01205234144500544</v>
+        <v>0.118728239714194</v>
       </c>
       <c r="G44" s="4" t="n">
-        <v>16.6322311941075</v>
+        <v>163.8449708055877</v>
       </c>
       <c r="H44" s="4" t="n">
         <v>57.69640916767813</v>
@@ -3210,10 +3210,10 @@
         <v>22</v>
       </c>
       <c r="F45" s="4" t="n">
-        <v>0.01316912353193327</v>
+        <v>0.1242152229968221</v>
       </c>
       <c r="G45" s="4" t="n">
-        <v>18.17339047406791</v>
+        <v>171.4170077356144</v>
       </c>
       <c r="H45" s="4" t="n">
         <v>57.62012634609287</v>
@@ -3271,10 +3271,10 @@
         <v>23</v>
       </c>
       <c r="F46" s="4" t="n">
-        <v>0.01433537836227827</v>
+        <v>0.1297403478566832</v>
       </c>
       <c r="G46" s="4" t="n">
-        <v>19.78282213994402</v>
+        <v>179.0416800422229</v>
       </c>
       <c r="H46" s="4" t="n">
         <v>57.54994760024488</v>
@@ -3332,10 +3332,10 @@
         <v>19</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>0.01009220966334404</v>
+        <v>0.1092069941428878</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>13.92724933541477</v>
+        <v>150.7056519171852</v>
       </c>
       <c r="H47" s="4" t="n">
         <v>62.91249399161276</v>
@@ -3393,10 +3393,10 @@
         <v>20</v>
       </c>
       <c r="F48" s="4" t="n">
-        <v>0.01112281254152821</v>
+        <v>0.114696564809534</v>
       </c>
       <c r="G48" s="4" t="n">
-        <v>15.34948130730892</v>
+        <v>158.2812594371569</v>
       </c>
       <c r="H48" s="4" t="n">
         <v>62.8201474340242</v>
@@ -3454,10 +3454,10 @@
         <v>21</v>
       </c>
       <c r="F49" s="4" t="n">
-        <v>0.01220350867805338</v>
+        <v>0.1202173959552566</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>16.84084197571367</v>
+        <v>165.9000064182542</v>
       </c>
       <c r="H49" s="4" t="n">
         <v>62.73580549948707</v>
@@ -3515,10 +3515,10 @@
         <v>22</v>
       </c>
       <c r="F50" s="4" t="n">
-        <v>0.01333429807291956</v>
+        <v>0.1257732000628174</v>
       </c>
       <c r="G50" s="4" t="n">
-        <v>18.401331340629</v>
+        <v>173.567016086688</v>
       </c>
       <c r="H50" s="4" t="n">
         <v>62.65847818265598</v>
@@ -3576,10 +3576,10 @@
         <v>23</v>
       </c>
       <c r="F51" s="4" t="n">
-        <v>0.01451518072612676</v>
+        <v>0.131367624140687</v>
       </c>
       <c r="G51" s="4" t="n">
-        <v>20.03094940205492</v>
+        <v>181.287321314148</v>
       </c>
       <c r="H51" s="4" t="n">
         <v>62.58733114000648</v>
@@ -3637,10 +3637,10 @@
         <v>19</v>
       </c>
       <c r="F52" s="4" t="n">
-        <v>0.04429163229331472</v>
+        <v>0.2334133140213605</v>
       </c>
       <c r="G52" s="4" t="n">
-        <v>61.12245256477431</v>
+        <v>322.1103733494775</v>
       </c>
       <c r="H52" s="4" t="n">
         <v>41.5299257828009</v>
@@ -3698,10 +3698,10 @@
         <v>20</v>
       </c>
       <c r="F53" s="4" t="n">
-        <v>0.048814634216943</v>
+        <v>0.2451464350720125</v>
       </c>
       <c r="G53" s="4" t="n">
-        <v>67.36419521938134</v>
+        <v>338.3020803993772</v>
       </c>
       <c r="H53" s="4" t="n">
         <v>41.46849859969493</v>
@@ -3759,10 +3759,10 @@
         <v>21</v>
       </c>
       <c r="F54" s="4" t="n">
-        <v>0.05355748018393005</v>
+        <v>0.2569463706346505</v>
       </c>
       <c r="G54" s="4" t="n">
-        <v>73.90932265382347</v>
+        <v>354.5859914758178</v>
       </c>
       <c r="H54" s="4" t="n">
         <v>41.41259523426168</v>
@@ -3820,10 +3820,10 @@
         <v>22</v>
       </c>
       <c r="F55" s="4" t="n">
-        <v>0.05852017019427584</v>
+        <v>0.2688210555756396</v>
       </c>
       <c r="G55" s="4" t="n">
-        <v>80.75783486810066</v>
+        <v>370.9730566943827</v>
       </c>
       <c r="H55" s="4" t="n">
         <v>41.36150510045378</v>
@@ -3881,10 +3881,10 @@
         <v>23</v>
       </c>
       <c r="F56" s="4" t="n">
-        <v>0.06370270424798041</v>
+        <v>0.280778284820022</v>
       </c>
       <c r="G56" s="4" t="n">
-        <v>87.90973186221296</v>
+        <v>387.4740330516304</v>
       </c>
       <c r="H56" s="4" t="n">
         <v>41.31463410708209</v>
@@ -3942,10 +3942,10 @@
         <v>19</v>
       </c>
       <c r="F57" s="4" t="n">
-        <v>0.04266192790956361</v>
+        <v>0.2365211920210906</v>
       </c>
       <c r="G57" s="4" t="n">
-        <v>58.87346051519778</v>
+        <v>326.3992449891051</v>
       </c>
       <c r="H57" s="4" t="n">
         <v>46.56207810171846</v>
@@ -4003,10 +4003,10 @@
         <v>20</v>
       </c>
       <c r="F58" s="4" t="n">
-        <v>0.0470185066132519</v>
+        <v>0.2484105385592834</v>
       </c>
       <c r="G58" s="4" t="n">
-        <v>64.88553912628761</v>
+        <v>342.8065432118112</v>
       </c>
       <c r="H58" s="4" t="n">
         <v>46.49963371217726</v>
@@ -4064,10 +4064,10 @@
         <v>21</v>
       </c>
       <c r="F59" s="4" t="n">
-        <v>0.05158684022962905</v>
+        <v>0.2603675892388851</v>
       </c>
       <c r="G59" s="4" t="n">
-        <v>71.1898395168881</v>
+        <v>359.3072731496615</v>
       </c>
       <c r="H59" s="4" t="n">
         <v>46.44280166228347</v>
@@ -4125,10 +4125,10 @@
         <v>22</v>
       </c>
       <c r="F60" s="4" t="n">
-        <v>0.05636692875869508</v>
+        <v>0.2724003845783173</v>
       </c>
       <c r="G60" s="4" t="n">
-        <v>77.78636168699921</v>
+        <v>375.9125307180778</v>
       </c>
       <c r="H60" s="4" t="n">
         <v>46.39086042718279</v>
@@ -4186,10 +4186,10 @@
         <v>23</v>
       </c>
       <c r="F61" s="4" t="n">
-        <v>0.06135877220044998</v>
+        <v>0.2845168232913718</v>
       </c>
       <c r="G61" s="4" t="n">
-        <v>84.67510563662097</v>
+        <v>392.6332161420931</v>
       </c>
       <c r="H61" s="4" t="n">
         <v>46.34320668658913</v>
@@ -4247,10 +4247,10 @@
         <v>19</v>
       </c>
       <c r="F62" s="4" t="n">
-        <v>0.04112717155433831</v>
+        <v>0.2396072900136138</v>
       </c>
       <c r="G62" s="4" t="n">
-        <v>56.75549674498686</v>
+        <v>330.6580602187871</v>
       </c>
       <c r="H62" s="4" t="n">
         <v>51.59405768456005</v>
@@ -4308,10 +4308,10 @@
         <v>20</v>
       </c>
       <c r="F63" s="4" t="n">
-        <v>0.0453270230030676</v>
+        <v>0.2516517672112218</v>
       </c>
       <c r="G63" s="4" t="n">
-        <v>62.55129174423329</v>
+        <v>347.2794387514862</v>
       </c>
       <c r="H63" s="4" t="n">
         <v>51.53060070369799</v>
@@ -4369,10 +4369,10 @@
         <v>21</v>
       </c>
       <c r="F64" s="4" t="n">
-        <v>0.04973101151377145</v>
+        <v>0.2637648319451394</v>
       </c>
       <c r="G64" s="4" t="n">
-        <v>68.62879588900459</v>
+        <v>363.9954680842924</v>
       </c>
       <c r="H64" s="4" t="n">
         <v>51.47284400816587</v>
@@ -4430,10 +4430,10 @@
         <v>22</v>
       </c>
       <c r="F65" s="4" t="n">
-        <v>0.05433913708644986</v>
+        <v>0.2759546296454347</v>
       </c>
       <c r="G65" s="4" t="n">
-        <v>74.9880091793008</v>
+        <v>380.8173889106999</v>
       </c>
       <c r="H65" s="4" t="n">
         <v>51.42005523138261</v>
@@ -4491,10 +4491,10 @@
         <v>23</v>
       </c>
       <c r="F66" s="4" t="n">
-        <v>0.05915139972110284</v>
+        <v>0.2882291620872979</v>
       </c>
       <c r="G66" s="4" t="n">
-        <v>81.62893161512193</v>
+        <v>397.7562436804711</v>
       </c>
       <c r="H66" s="4" t="n">
         <v>51.37162190108249</v>
@@ -4552,10 +4552,10 @@
         <v>19</v>
       </c>
       <c r="F67" s="4" t="n">
-        <v>0.03968015987234906</v>
+        <v>0.2426720082487107</v>
       </c>
       <c r="G67" s="4" t="n">
-        <v>54.7586206238417</v>
+        <v>334.8873713832207</v>
       </c>
       <c r="H67" s="4" t="n">
         <v>56.62586419648375</v>
@@ -4613,10 +4613,10 @@
         <v>20</v>
       </c>
       <c r="F68" s="4" t="n">
-        <v>0.04373224443414566</v>
+        <v>0.2548705413971942</v>
       </c>
       <c r="G68" s="4" t="n">
-        <v>60.35049731912101</v>
+        <v>351.7213471281279</v>
       </c>
       <c r="H68" s="4" t="n">
         <v>56.56139934910909</v>
@@ -4674,10 +4674,10 @@
         <v>21</v>
       </c>
       <c r="F69" s="4" t="n">
-        <v>0.04798128373289324</v>
+        <v>0.2671385393569364</v>
       </c>
       <c r="G69" s="4" t="n">
-        <v>66.21417155139267</v>
+        <v>368.6511843125723</v>
       </c>
       <c r="H69" s="4" t="n">
         <v>56.50272214606497</v>
@@ -4735,10 +4735,10 @@
         <v>22</v>
       </c>
       <c r="F70" s="4" t="n">
-        <v>0.05242727776859181</v>
+        <v>0.2794842517428496</v>
       </c>
       <c r="G70" s="4" t="n">
-        <v>72.3496433206567</v>
+        <v>385.6882674051324</v>
       </c>
       <c r="H70" s="4" t="n">
         <v>56.4490894774645</v>
@@ -4796,10 +4796,10 @@
         <v>23</v>
       </c>
       <c r="F71" s="4" t="n">
-        <v>0.05707022654124135</v>
+        <v>0.2919157826775373</v>
       </c>
       <c r="G71" s="4" t="n">
-        <v>78.75691262691306</v>
+        <v>402.8437800950014</v>
       </c>
       <c r="H71" s="4" t="n">
         <v>56.39987979731251</v>
@@ -4857,10 +4857,10 @@
         <v>19</v>
       </c>
       <c r="F72" s="4" t="n">
-        <v>0.03831435140271525</v>
+        <v>0.2457157368214976</v>
       </c>
       <c r="G72" s="4" t="n">
-        <v>52.87380493574704</v>
+        <v>339.0877168136666</v>
       </c>
       <c r="H72" s="4" t="n">
         <v>61.65749724103617</v>
@@ -4918,10 +4918,10 @@
         <v>20</v>
       </c>
       <c r="F73" s="4" t="n">
-        <v>0.04222696144041773</v>
+        <v>0.2580672708214515</v>
       </c>
       <c r="G73" s="4" t="n">
-        <v>58.27320678777647</v>
+        <v>356.1328337336031</v>
       </c>
       <c r="H73" s="4" t="n">
         <v>61.5920293589661</v>
@@ -4979,10 +4979,10 @@
         <v>21</v>
       </c>
       <c r="F74" s="4" t="n">
-        <v>0.04632974694682411</v>
+        <v>0.2704891408993275</v>
       </c>
       <c r="G74" s="4" t="n">
-        <v>63.93505078661727</v>
+        <v>373.2750144410719</v>
       </c>
       <c r="H74" s="4" t="n">
         <v>61.53243588355073</v>
@@ -5040,10 +5040,10 @@
         <v>22</v>
       </c>
       <c r="F75" s="4" t="n">
-        <v>0.05062270792193437</v>
+        <v>0.2829897001413391</v>
       </c>
       <c r="G75" s="4" t="n">
-        <v>69.85933693226943</v>
+        <v>390.525786195048</v>
       </c>
       <c r="H75" s="4" t="n">
         <v>61.47796306128672</v>
@@ -5101,10 +5101,10 @@
         <v>23</v>
       </c>
       <c r="F76" s="4" t="n">
-        <v>0.05510584436574853</v>
+        <v>0.2955771543165457</v>
       </c>
       <c r="G76" s="4" t="n">
-        <v>76.04606522473297</v>
+        <v>407.8964729568331</v>
       </c>
       <c r="H76" s="4" t="n">
         <v>61.42798035177444</v>
@@ -5162,10 +5162,10 @@
         <v>19</v>
       </c>
       <c r="F77" s="4" t="n">
-        <v>0.1087089054406912</v>
+        <v>0.4149570027046409</v>
       </c>
       <c r="G77" s="4" t="n">
-        <v>150.0182895081538</v>
+        <v>572.6406637324045</v>
       </c>
       <c r="H77" s="4" t="n">
         <v>40.85076206583437</v>
@@ -5223,10 +5223,10 @@
         <v>20</v>
       </c>
       <c r="F78" s="4" t="n">
-        <v>0.1198101126657405</v>
+        <v>0.4358158845724666</v>
       </c>
       <c r="G78" s="4" t="n">
-        <v>165.3379554787219</v>
+        <v>601.4259207100039</v>
       </c>
       <c r="H78" s="4" t="n">
         <v>40.80476255539014</v>
@@ -5284,10 +5284,10 @@
         <v>21</v>
       </c>
       <c r="F79" s="4" t="n">
-        <v>0.1314509027438876</v>
+        <v>0.4567935477949341</v>
       </c>
       <c r="G79" s="4" t="n">
-        <v>181.4022457865649</v>
+        <v>630.3750959570091</v>
       </c>
       <c r="H79" s="4" t="n">
         <v>40.76294111905883</v>
@@ -5345,10 +5345,10 @@
         <v>22</v>
       </c>
       <c r="F80" s="4" t="n">
-        <v>0.1436312756751325</v>
+        <v>0.4779040988011372</v>
       </c>
       <c r="G80" s="4" t="n">
-        <v>198.2111604316829</v>
+        <v>659.5076563455693</v>
       </c>
       <c r="H80" s="4" t="n">
         <v>40.72475416993797</v>
@@ -5406,10 +5406,10 @@
         <v>23</v>
       </c>
       <c r="F81" s="4" t="n">
-        <v>0.1563512314594753</v>
+        <v>0.4991613952355948</v>
       </c>
       <c r="G81" s="4" t="n">
-        <v>215.7646994140759</v>
+        <v>688.8427254251208</v>
       </c>
       <c r="H81" s="4" t="n">
         <v>40.68974835378247</v>
@@ -5467,10 +5467,10 @@
         <v>19</v>
       </c>
       <c r="F82" s="4" t="n">
-        <v>0.1076904467640727</v>
+        <v>0.4204821191486057</v>
       </c>
       <c r="G82" s="4" t="n">
-        <v>148.6128165344204</v>
+        <v>580.2653244250758</v>
       </c>
       <c r="H82" s="4" t="n">
         <v>45.87593289838563</v>
@@ -5528,10 +5528,10 @@
         <v>20</v>
       </c>
       <c r="F83" s="4" t="n">
-        <v>0.1186876503587528</v>
+        <v>0.4416187352165039</v>
       </c>
       <c r="G83" s="4" t="n">
-        <v>163.7889574950789</v>
+        <v>609.4338545987753</v>
       </c>
       <c r="H83" s="4" t="n">
         <v>45.82913186321786</v>
@@ -5589,10 +5589,10 @@
         <v>21</v>
       </c>
       <c r="F84" s="4" t="n">
-        <v>0.1302193816287947</v>
+        <v>0.4628757142024625</v>
       </c>
       <c r="G84" s="4" t="n">
-        <v>179.7027466477367</v>
+        <v>638.7684855993982</v>
       </c>
       <c r="H84" s="4" t="n">
         <v>45.78658112685925</v>
@@ -5650,10 +5650,10 @@
         <v>22</v>
       </c>
       <c r="F85" s="4" t="n">
-        <v>0.1422856405741985</v>
+        <v>0.484267350361453</v>
       </c>
       <c r="G85" s="4" t="n">
-        <v>196.3541839923939</v>
+        <v>668.2889434988051</v>
       </c>
       <c r="H85" s="4" t="n">
         <v>45.7477278184323</v>
@@ -5711,10 +5711,10 @@
         <v>23</v>
       </c>
       <c r="F86" s="4" t="n">
-        <v>0.154886427194964</v>
+        <v>0.5058076858513278</v>
       </c>
       <c r="G86" s="4" t="n">
-        <v>213.7432695290503</v>
+        <v>698.0146064748325</v>
       </c>
       <c r="H86" s="4" t="n">
         <v>45.71211081650298</v>
@@ -5772,10 +5772,10 @@
         <v>19</v>
       </c>
       <c r="F87" s="4" t="n">
-        <v>0.1066972564059439</v>
+        <v>0.425968515579758</v>
       </c>
       <c r="G87" s="4" t="n">
-        <v>147.2422138402025</v>
+        <v>587.836551500066</v>
       </c>
       <c r="H87" s="4" t="n">
         <v>50.90099014480675</v>
@@ -5833,10 +5833,10 @@
         <v>20</v>
       </c>
       <c r="F88" s="4" t="n">
-        <v>0.1175930367369565</v>
+        <v>0.4473809194866166</v>
       </c>
       <c r="G88" s="4" t="n">
-        <v>162.2783906969999</v>
+        <v>617.3856688915309</v>
       </c>
       <c r="H88" s="4" t="n">
         <v>50.85338934315983</v>
@@ -5894,10 +5894,10 @@
         <v>21</v>
       </c>
       <c r="F89" s="4" t="n">
-        <v>0.1290184149863351</v>
+        <v>0.4689152567913589</v>
       </c>
       <c r="G89" s="4" t="n">
-        <v>178.0454126811424</v>
+        <v>647.1030543720753</v>
       </c>
       <c r="H89" s="4" t="n">
         <v>50.8101108441414</v>
@@ -5955,10 +5955,10 @@
         <v>22</v>
       </c>
       <c r="F90" s="4" t="n">
-        <v>0.1409733911540796</v>
+        <v>0.4905860082585505</v>
       </c>
       <c r="G90" s="4" t="n">
-        <v>194.5432797926299</v>
+        <v>677.0086913967997</v>
       </c>
       <c r="H90" s="4" t="n">
         <v>50.77059253126589</v>
@@ -6016,10 +6016,10 @@
         <v>23</v>
       </c>
       <c r="F91" s="4" t="n">
-        <v>0.1534579652401901</v>
+        <v>0.5124073992663074</v>
       </c>
       <c r="G91" s="4" t="n">
-        <v>211.7719920314624</v>
+        <v>707.1222109875042</v>
       </c>
       <c r="H91" s="4" t="n">
         <v>50.73436554607486</v>
@@ -6077,10 +6077,10 @@
         <v>19</v>
       </c>
       <c r="F92" s="4" t="n">
-        <v>0.1057283141730603</v>
+        <v>0.4314169035532635</v>
       </c>
       <c r="G92" s="4" t="n">
-        <v>145.9050735588232</v>
+        <v>595.3553269035035</v>
       </c>
       <c r="H92" s="4" t="n">
         <v>55.92593357523681</v>
@@ -6138,10 +6138,10 @@
         <v>20</v>
       </c>
       <c r="F93" s="4" t="n">
-        <v>0.1165251474263451</v>
+        <v>0.4531031847061229</v>
       </c>
       <c r="G93" s="4" t="n">
-        <v>160.8047034483563</v>
+        <v>625.2823948944497</v>
       </c>
       <c r="H93" s="4" t="n">
         <v>55.87753486009973</v>
@@ -6199,10 +6199,10 @@
         <v>21</v>
       </c>
       <c r="F94" s="4" t="n">
-        <v>0.1278467691979529</v>
+        <v>0.4749129588567759</v>
       </c>
       <c r="G94" s="4" t="n">
-        <v>176.428541493175</v>
+        <v>655.3798832223508</v>
       </c>
       <c r="H94" s="4" t="n">
         <v>55.83353022056945</v>
@@ -6260,10 +6260,10 @@
         <v>22</v>
       </c>
       <c r="F95" s="4" t="n">
-        <v>0.1396931794878836</v>
+        <v>0.4968608919872883</v>
       </c>
       <c r="G95" s="4" t="n">
-        <v>192.7765876932794</v>
+        <v>685.6680309424578</v>
       </c>
       <c r="H95" s="4" t="n">
         <v>55.79334833438535</v>
@@ -6321,10 +6321,10 @@
         <v>23</v>
       </c>
       <c r="F96" s="4" t="n">
-        <v>0.1520643782961372</v>
+        <v>0.5189613914267329</v>
       </c>
       <c r="G96" s="4" t="n">
-        <v>209.8488420486693</v>
+        <v>716.1667201688914</v>
       </c>
       <c r="H96" s="4" t="n">
         <v>55.75651263742603</v>
@@ -6382,10 +6382,10 @@
         <v>19</v>
       </c>
       <c r="F97" s="4" t="n">
-        <v>0.1047826570182218</v>
+        <v>0.4368279765715511</v>
       </c>
       <c r="G97" s="4" t="n">
-        <v>144.6000666851461</v>
+        <v>602.8226076687406</v>
       </c>
       <c r="H97" s="4" t="n">
         <v>60.95076288956206</v>
@@ -6443,10 +6443,10 @@
         <v>20</v>
       </c>
       <c r="F98" s="4" t="n">
-        <v>0.1154829210346336</v>
+        <v>0.458786259238136</v>
       </c>
       <c r="G98" s="4" t="n">
-        <v>159.3664310277944</v>
+        <v>633.1250377486277</v>
       </c>
       <c r="H98" s="4" t="n">
         <v>60.90156820790674</v>
@@ -6504,10 +6504,10 @@
         <v>21</v>
       </c>
       <c r="F99" s="4" t="n">
-        <v>0.1267032797461384</v>
+        <v>0.4808695838210266</v>
       </c>
       <c r="G99" s="4" t="n">
-        <v>174.8505260496709</v>
+        <v>663.6000256730167</v>
       </c>
       <c r="H99" s="4" t="n">
         <v>60.85683913417407</v>
@@ -6565,10 +6565,10 @@
         <v>22</v>
       </c>
       <c r="F100" s="4" t="n">
-        <v>0.1384437331527361</v>
+        <v>0.5030928002512695</v>
       </c>
       <c r="G100" s="4" t="n">
-        <v>191.0523517507758</v>
+        <v>694.2680643467519</v>
       </c>
       <c r="H100" s="4" t="n">
         <v>60.81599518159774</v>
@@ -6626,10 +6626,10 @@
         <v>23</v>
       </c>
       <c r="F101" s="4" t="n">
-        <v>0.1507042812544267</v>
+        <v>0.5254704965627479</v>
       </c>
       <c r="G101" s="4" t="n">
-        <v>207.9719081311089</v>
+        <v>725.1492852565921</v>
       </c>
       <c r="H101" s="4" t="n">
         <v>60.77855211292835</v>
@@ -6687,10 +6687,10 @@
         <v>19</v>
       </c>
       <c r="F102" s="4" t="n">
-        <v>0.2008018264540105</v>
+        <v>0.6483703167260015</v>
       </c>
       <c r="G102" s="4" t="n">
-        <v>277.1065205065345</v>
+        <v>894.7510370818821</v>
       </c>
       <c r="H102" s="4" t="n">
         <v>40.4220125621817</v>
@@ -6748,10 +6748,10 @@
         <v>20</v>
       </c>
       <c r="F103" s="4" t="n">
-        <v>0.2213074389206038</v>
+        <v>0.6809623196444792</v>
       </c>
       <c r="G103" s="4" t="n">
-        <v>305.4042657104332</v>
+        <v>939.7280011093812</v>
       </c>
       <c r="H103" s="4" t="n">
         <v>40.38570860899471</v>
@@ -6809,10 +6809,10 @@
         <v>21</v>
       </c>
       <c r="F104" s="4" t="n">
-        <v>0.2428097427068832</v>
+        <v>0.7137399184295846</v>
       </c>
       <c r="G104" s="4" t="n">
-        <v>335.0774449354988</v>
+        <v>984.9610874328267</v>
       </c>
       <c r="H104" s="4" t="n">
         <v>40.35270994378514</v>
@@ -6870,10 +6870,10 @@
         <v>22</v>
       </c>
       <c r="F105" s="4" t="n">
-        <v>0.2653087378128487</v>
+        <v>0.7467251543767768</v>
       </c>
       <c r="G105" s="4" t="n">
-        <v>366.1260581817312</v>
+        <v>1030.480713039952</v>
       </c>
       <c r="H105" s="4" t="n">
         <v>40.32258514083467</v>
@@ -6931,10 +6931,10 @@
         <v>23</v>
       </c>
       <c r="F106" s="4" t="n">
-        <v>0.2888044242385002</v>
+        <v>0.7799396800556169</v>
       </c>
       <c r="G106" s="4" t="n">
-        <v>398.5501054491302</v>
+        <v>1076.316758476751</v>
       </c>
       <c r="H106" s="4" t="n">
         <v>40.29497467449837</v>
@@ -6992,10 +6992,10 @@
         <v>19</v>
       </c>
       <c r="F107" s="4" t="n">
-        <v>0.1989205789002441</v>
+        <v>0.6570033111696963</v>
       </c>
       <c r="G107" s="4" t="n">
-        <v>274.5103988823369</v>
+        <v>906.664569414181</v>
       </c>
       <c r="H107" s="4" t="n">
         <v>45.44252976278711</v>
@@ -7053,10 +7053,10 @@
         <v>20</v>
       </c>
       <c r="F108" s="4" t="n">
-        <v>0.2192340808966665</v>
+        <v>0.6900292737757872</v>
       </c>
       <c r="G108" s="4" t="n">
-        <v>302.5430316373998</v>
+        <v>952.2403978105863</v>
       </c>
       <c r="H108" s="4" t="n">
         <v>45.40558250510281</v>
@@ -7114,10 +7114,10 @@
         <v>21</v>
       </c>
       <c r="F109" s="4" t="n">
-        <v>0.2405349365332324</v>
+        <v>0.7232433034413476</v>
       </c>
       <c r="G109" s="4" t="n">
-        <v>331.9382124158606</v>
+        <v>998.0757587490597</v>
       </c>
       <c r="H109" s="4" t="n">
         <v>45.3719992732551</v>
@@ -7175,10 +7175,10 @@
         <v>22</v>
       </c>
       <c r="F110" s="4" t="n">
-        <v>0.2628231458099414</v>
+        <v>0.7566677349397705</v>
       </c>
       <c r="G110" s="4" t="n">
-        <v>362.6959412177192</v>
+        <v>1044.201474216883</v>
       </c>
       <c r="H110" s="4" t="n">
         <v>45.34134097259905</v>
@@ -7236,10 +7236,10 @@
         <v>23</v>
       </c>
       <c r="F111" s="4" t="n">
-        <v>0.2860987087267939</v>
+        <v>0.7903245091426997</v>
       </c>
       <c r="G111" s="4" t="n">
-        <v>394.8162180429756</v>
+        <v>1090.647822616926</v>
       </c>
       <c r="H111" s="4" t="n">
         <v>45.31324168394944</v>
@@ -7297,10 +7297,10 @@
         <v>19</v>
       </c>
       <c r="F112" s="4" t="n">
-        <v>0.1970860057609018</v>
+        <v>0.6655758055933718</v>
       </c>
       <c r="G112" s="4" t="n">
-        <v>271.9786879500445</v>
+        <v>918.4946117188531</v>
       </c>
       <c r="H112" s="4" t="n">
         <v>50.46295956130928</v>
@@ -7358,10 +7358,10 @@
         <v>20</v>
       </c>
       <c r="F113" s="4" t="n">
-        <v>0.2172121636155836</v>
+        <v>0.6990326866978386</v>
       </c>
       <c r="G113" s="4" t="n">
-        <v>299.7527857895054</v>
+        <v>964.6651076430172</v>
       </c>
       <c r="H113" s="4" t="n">
         <v>50.42536968582122</v>
@@ -7419,10 +7419,10 @@
         <v>21</v>
       </c>
       <c r="F114" s="4" t="n">
-        <v>0.2383165691019844</v>
+        <v>0.7326800887364984</v>
       </c>
       <c r="G114" s="4" t="n">
-        <v>328.8768653607385</v>
+        <v>1011.098522456368</v>
       </c>
       <c r="H114" s="4" t="n">
         <v>50.39120249471908</v>
@@ -7480,10 +7480,10 @@
         <v>22</v>
       </c>
       <c r="F115" s="4" t="n">
-        <v>0.2603992222201042</v>
+        <v>0.7665406379039854</v>
       </c>
       <c r="G115" s="4" t="n">
-        <v>359.3509266637438</v>
+        <v>1057.8260803075</v>
       </c>
       <c r="H115" s="4" t="n">
         <v>50.36001123802519</v>
@@ -7541,10 +7541,10 @@
         <v>23</v>
       </c>
       <c r="F116" s="4" t="n">
-        <v>0.2834601229699431</v>
+        <v>0.8006365613536055</v>
       </c>
       <c r="G116" s="4" t="n">
-        <v>391.1749696985214</v>
+        <v>1104.878454667976</v>
       </c>
       <c r="H116" s="4" t="n">
         <v>50.33142361364603</v>
@@ -7602,10 +7602,10 @@
         <v>19</v>
       </c>
       <c r="F117" s="4" t="n">
-        <v>0.1952962225844205</v>
+        <v>0.6740889118019743</v>
       </c>
       <c r="G117" s="4" t="n">
-        <v>269.5087871665003</v>
+        <v>930.2426982867245</v>
       </c>
       <c r="H117" s="4" t="n">
         <v>55.48330197582109</v>
@@ -7663,10 +7663,10 @@
         <v>20</v>
       </c>
       <c r="F118" s="4" t="n">
-        <v>0.2152396101881327</v>
+        <v>0.7079737261033173</v>
       </c>
       <c r="G118" s="4" t="n">
-        <v>297.0306620596231</v>
+        <v>977.0037420225779</v>
       </c>
       <c r="H118" s="4" t="n">
         <v>55.44507023928743</v>
@@ -7724,10 +7724,10 @@
         <v>21</v>
       </c>
       <c r="F119" s="4" t="n">
-        <v>0.2361523617326751</v>
+        <v>0.7420514982137125</v>
       </c>
       <c r="G119" s="4" t="n">
-        <v>325.8902591910917</v>
+        <v>1024.031067534923</v>
       </c>
       <c r="H119" s="4" t="n">
         <v>55.41031975890269</v>
@@ -7785,10 +7785,10 @@
         <v>22</v>
       </c>
       <c r="F120" s="4" t="n">
-        <v>0.2580344772180478</v>
+        <v>0.7763451437301381</v>
       </c>
       <c r="G120" s="4" t="n">
-        <v>356.087578560906</v>
+        <v>1071.356298347591</v>
       </c>
       <c r="H120" s="4" t="n">
         <v>55.37859614407977</v>
@@ -7846,10 +7846,10 @@
         <v>23</v>
       </c>
       <c r="F121" s="4" t="n">
-        <v>0.2808859566442507</v>
+        <v>0.8108771741042703</v>
       </c>
       <c r="G121" s="4" t="n">
-        <v>387.622620169066</v>
+        <v>1119.010500263893</v>
       </c>
       <c r="H121" s="4" t="n">
         <v>55.34952072136148</v>
@@ -7907,10 +7907,10 @@
         <v>19</v>
       </c>
       <c r="F122" s="4" t="n">
-        <v>0.1935494504766425</v>
+        <v>0.6825437133930488</v>
       </c>
       <c r="G122" s="4" t="n">
-        <v>267.0982416577667</v>
+        <v>941.9103244824073</v>
       </c>
       <c r="H122" s="4" t="n">
         <v>60.50355695363334</v>
@@ -7968,10 +7968,10 @@
         <v>20</v>
       </c>
       <c r="F123" s="4" t="n">
-        <v>0.2133144600618771</v>
+        <v>0.7168535300595877</v>
       </c>
       <c r="G123" s="4" t="n">
-        <v>294.3739548853904</v>
+        <v>989.2578714822311</v>
       </c>
       <c r="H123" s="4" t="n">
         <v>60.46468418302845</v>
@@ -8029,10 +8029,10 @@
         <v>21</v>
       </c>
       <c r="F124" s="4" t="n">
-        <v>0.2340401633849462</v>
+        <v>0.751358724720354</v>
       </c>
       <c r="G124" s="4" t="n">
-        <v>322.9754254712257</v>
+        <v>1036.875040114089</v>
       </c>
       <c r="H124" s="4" t="n">
         <v>60.42935114608579</v>
@@ -8090,10 +8090,10 @@
         <v>22</v>
       </c>
       <c r="F125" s="4" t="n">
-        <v>0.2557265604458495</v>
+        <v>0.7860825003926086</v>
       </c>
       <c r="G125" s="4" t="n">
-        <v>352.9026534152723</v>
+        <v>1084.7938505418</v>
       </c>
       <c r="H125" s="4" t="n">
         <v>60.3970958274529</v>
@@ -8151,10 +8151,10 @@
         <v>23</v>
       </c>
       <c r="F126" s="4" t="n">
-        <v>0.2783736512445874</v>
+        <v>0.8210476508792939</v>
       </c>
       <c r="G126" s="4" t="n">
-        <v>384.1556387175306</v>
+        <v>1133.045758213426</v>
       </c>
       <c r="H126" s="4" t="n">
         <v>60.36753319476461</v>
@@ -8212,10 +8212,10 @@
         <v>19</v>
       </c>
       <c r="F127" s="4" t="n">
-        <v>0.6123766479042156</v>
+        <v>1.458833212633503</v>
       </c>
       <c r="G127" s="4" t="n">
-        <v>845.0797741078176</v>
+        <v>2013.189833434234</v>
       </c>
       <c r="H127" s="4" t="n">
         <v>39.82490672252924</v>
@@ -8273,10 +8273,10 @@
         <v>20</v>
       </c>
       <c r="F128" s="4" t="n">
-        <v>0.6749117276256705</v>
+        <v>1.532165219200078</v>
       </c>
       <c r="G128" s="4" t="n">
-        <v>931.3781841234253</v>
+        <v>2114.388002496108</v>
       </c>
       <c r="H128" s="4" t="n">
         <v>39.80145673342437</v>
@@ -8334,10 +8334,10 @@
         <v>21</v>
       </c>
       <c r="F129" s="4" t="n">
-        <v>0.7404863737700155</v>
+        <v>1.605914816466565</v>
       </c>
       <c r="G129" s="4" t="n">
-        <v>1021.871195802621</v>
+        <v>2216.16244672386</v>
       </c>
       <c r="H129" s="4" t="n">
         <v>39.7801372865006</v>
@@ -8395,10 +8395,10 @@
         <v>22</v>
       </c>
       <c r="F130" s="4" t="n">
-        <v>0.8091005863372506</v>
+        <v>1.680131597347748</v>
       </c>
       <c r="G130" s="4" t="n">
-        <v>1116.558809145406</v>
+        <v>2318.581604339892</v>
       </c>
       <c r="H130" s="4" t="n">
         <v>39.76067063220303</v>
@@ -8456,10 +8456,10 @@
         <v>23</v>
       </c>
       <c r="F131" s="4" t="n">
-        <v>0.8807543653273754</v>
+        <v>1.754864280125138</v>
       </c>
       <c r="G131" s="4" t="n">
-        <v>1215.441024151778</v>
+        <v>2421.71270657269</v>
       </c>
       <c r="H131" s="4" t="n">
         <v>39.74282528991564</v>
@@ -8517,10 +8517,10 @@
         <v>19</v>
       </c>
       <c r="F132" s="4" t="n">
-        <v>0.6066394885805316</v>
+        <v>1.478257450131817</v>
       </c>
       <c r="G132" s="4" t="n">
-        <v>837.1624942411337</v>
+        <v>2039.995281181907</v>
       </c>
       <c r="H132" s="4" t="n">
         <v>44.83893801028123</v>
@@ -8578,10 +8578,10 @@
         <v>20</v>
       </c>
       <c r="F133" s="4" t="n">
-        <v>0.6685886973075436</v>
+        <v>1.552565865995522</v>
       </c>
       <c r="G133" s="4" t="n">
-        <v>922.6524022844101</v>
+        <v>2142.54089507382</v>
       </c>
       <c r="H133" s="4" t="n">
         <v>44.81507339349512</v>
@@ -8639,10 +8639,10 @@
         <v>21</v>
       </c>
       <c r="F134" s="4" t="n">
-        <v>0.733548995739885</v>
+        <v>1.627297432743032</v>
       </c>
       <c r="G134" s="4" t="n">
-        <v>1012.297614121041</v>
+        <v>2245.670457185385</v>
       </c>
       <c r="H134" s="4" t="n">
         <v>44.79337731684114</v>
@@ -8700,10 +8700,10 @@
         <v>22</v>
       </c>
       <c r="F135" s="4" t="n">
-        <v>0.801520383877556</v>
+        <v>1.702502403614484</v>
       </c>
       <c r="G135" s="4" t="n">
-        <v>1106.098129751027</v>
+        <v>2349.453316987988</v>
       </c>
       <c r="H135" s="4" t="n">
         <v>44.77356703786459</v>
@@ -8761,10 +8761,10 @@
         <v>23</v>
       </c>
       <c r="F136" s="4" t="n">
-        <v>0.8725028617205561</v>
+        <v>1.778230145571075</v>
       </c>
       <c r="G136" s="4" t="n">
-        <v>1204.053949174368</v>
+        <v>2453.957600888083</v>
       </c>
       <c r="H136" s="4" t="n">
         <v>44.75540692076859</v>
@@ -8822,10 +8822,10 @@
         <v>19</v>
       </c>
       <c r="F137" s="4" t="n">
-        <v>0.6010446702004165</v>
+        <v>1.497545562585086</v>
       </c>
       <c r="G137" s="4" t="n">
-        <v>829.4416448765747</v>
+        <v>2066.612876367419</v>
       </c>
       <c r="H137" s="4" t="n">
         <v>49.85290586071058</v>
@@ -8883,10 +8883,10 @@
         <v>20</v>
       </c>
       <c r="F138" s="4" t="n">
-        <v>0.6624225435987139</v>
+        <v>1.572823545070137</v>
       </c>
       <c r="G138" s="4" t="n">
-        <v>914.1431101662251</v>
+        <v>2170.496492196788</v>
       </c>
       <c r="H138" s="4" t="n">
         <v>49.82862679236329</v>
@@ -8944,10 +8944,10 @@
         <v>21</v>
       </c>
       <c r="F139" s="4" t="n">
-        <v>0.7267837365021727</v>
+        <v>1.648530199657121</v>
       </c>
       <c r="G139" s="4" t="n">
-        <v>1002.961556372998</v>
+        <v>2274.971675526827</v>
       </c>
       <c r="H139" s="4" t="n">
         <v>49.80655425442678</v>
@@ -9005,10 +9005,10 @@
         <v>22</v>
       </c>
       <c r="F140" s="4" t="n">
-        <v>0.7941282489107936</v>
+        <v>1.724716435283967</v>
       </c>
       <c r="G140" s="4" t="n">
-        <v>1095.896983496895</v>
+        <v>2380.108680691875</v>
       </c>
       <c r="H140" s="4" t="n">
         <v>49.78640051168492</v>
@@ -9066,10 +9066,10 @@
         <v>23</v>
       </c>
       <c r="F141" s="4" t="n">
-        <v>0.8644560808245758</v>
+        <v>1.801432263045612</v>
       </c>
       <c r="G141" s="4" t="n">
-        <v>1192.949391537915</v>
+        <v>2485.976523002945</v>
       </c>
       <c r="H141" s="4" t="n">
         <v>49.76792577338134</v>
@@ -9127,10 +9127,10 @@
         <v>19</v>
       </c>
       <c r="F142" s="4" t="n">
-        <v>0.5955864458334187</v>
+        <v>1.516700051554442</v>
       </c>
       <c r="G142" s="4" t="n">
-        <v>821.9092952501178</v>
+        <v>2093.046071145131</v>
       </c>
       <c r="H142" s="4" t="n">
         <v>54.86681061211047</v>
@@ -9188,10 +9188,10 @@
         <v>20</v>
       </c>
       <c r="F143" s="4" t="n">
-        <v>0.6564069326999206</v>
+        <v>1.592940883732464</v>
       </c>
       <c r="G143" s="4" t="n">
-        <v>905.8415671258904</v>
+        <v>2198.2584195508</v>
       </c>
       <c r="H143" s="4" t="n">
         <v>54.84211730189674</v>
@@ -9249,10 +9249,10 @@
         <v>21</v>
       </c>
       <c r="F144" s="4" t="n">
-        <v>0.720183646863592</v>
+        <v>1.669615870980854</v>
       </c>
       <c r="G144" s="4" t="n">
-        <v>993.853432671757</v>
+        <v>2304.069901953578</v>
       </c>
       <c r="H144" s="4" t="n">
         <v>54.81966850134627</v>
@@ -9310,10 +9310,10 @@
         <v>22</v>
       </c>
       <c r="F145" s="4" t="n">
-        <v>0.7869165883244332</v>
+        <v>1.746776573392811</v>
       </c>
       <c r="G145" s="4" t="n">
-        <v>1085.944891887718</v>
+        <v>2410.551671282079</v>
       </c>
       <c r="H145" s="4" t="n">
         <v>54.79917148310373</v>
@@ -9371,10 +9371,10 @@
         <v>23</v>
       </c>
       <c r="F146" s="4" t="n">
-        <v>0.8566057570824439</v>
+        <v>1.824473641734609</v>
       </c>
       <c r="G146" s="4" t="n">
-        <v>1182.115944773773</v>
+        <v>2517.77362559376</v>
       </c>
       <c r="H146" s="4" t="n">
         <v>54.78038230206889</v>
@@ -9432,10 +9432,10 @@
         <v>19</v>
       </c>
       <c r="F147" s="4" t="n">
-        <v>0.5902593904629404</v>
+        <v>1.53572335513436</v>
       </c>
       <c r="G147" s="4" t="n">
-        <v>814.5579588388578</v>
+        <v>2119.298230085416</v>
       </c>
       <c r="H147" s="4" t="n">
         <v>59.88065254396589</v>
@@ -9493,10 +9493,10 @@
         <v>20</v>
       </c>
       <c r="F148" s="4" t="n">
-        <v>0.6505358855991672</v>
+        <v>1.612920442634073</v>
       </c>
       <c r="G148" s="4" t="n">
-        <v>897.7395221268507</v>
+        <v>2225.83021083502</v>
       </c>
       <c r="H148" s="4" t="n">
         <v>59.85554523567526</v>
@@ -9554,10 +9554,10 @@
         <v>21</v>
       </c>
       <c r="F149" s="4" t="n">
-        <v>0.713742166889368</v>
+        <v>1.690557130620797</v>
       </c>
       <c r="G149" s="4" t="n">
-        <v>984.9641903073278</v>
+        <v>2332.968840256699</v>
       </c>
       <c r="H149" s="4" t="n">
         <v>59.83272040186707</v>
@@ -9615,10 +9615,10 @@
         <v>22</v>
       </c>
       <c r="F150" s="4" t="n">
-        <v>0.7798782343335425</v>
+        <v>1.76868562588337</v>
       </c>
       <c r="G150" s="4" t="n">
-        <v>1076.231963380289</v>
+        <v>2440.78616371905</v>
       </c>
       <c r="H150" s="4" t="n">
         <v>59.81188032416019</v>
@@ -9676,10 +9676,10 @@
         <v>23</v>
       </c>
       <c r="F151" s="4" t="n">
-        <v>0.8489440879316907</v>
+        <v>1.847357214478411</v>
       </c>
       <c r="G151" s="4" t="n">
-        <v>1171.542841345733</v>
+        <v>2549.352955980208</v>
       </c>
       <c r="H151" s="4" t="n">
         <v>59.79277690412715</v>
@@ -9737,10 +9737,10 @@
         <v>19</v>
       </c>
       <c r="F152" s="4" t="n">
-        <v>1.350828288332608</v>
+        <v>2.593481266904006</v>
       </c>
       <c r="G152" s="4" t="n">
-        <v>1864.143037898999</v>
+        <v>3579.004148327529</v>
       </c>
       <c r="H152" s="4" t="n">
         <v>39.51119583829732</v>
@@ -9798,10 +9798,10 @@
         <v>20</v>
       </c>
       <c r="F153" s="4" t="n">
-        <v>1.488773056458529</v>
+        <v>2.723849278577917</v>
       </c>
       <c r="G153" s="4" t="n">
-        <v>2054.50681791277</v>
+        <v>3758.912004437525</v>
       </c>
       <c r="H153" s="4" t="n">
         <v>39.49393291024827</v>
@@ -9859,10 +9859,10 @@
         <v>21</v>
       </c>
       <c r="F154" s="4" t="n">
-        <v>1.633422737847159</v>
+        <v>2.854959673718338</v>
       </c>
       <c r="G154" s="4" t="n">
-        <v>2254.123378229079</v>
+        <v>3939.844349731307</v>
       </c>
       <c r="H154" s="4" t="n">
         <v>39.47823431019501</v>
@@ -9920,10 +9920,10 @@
         <v>22</v>
       </c>
       <c r="F155" s="4" t="n">
-        <v>1.784777332498497</v>
+        <v>2.986900617507107</v>
       </c>
       <c r="G155" s="4" t="n">
-        <v>2462.992718847926</v>
+        <v>4121.922852159808</v>
       </c>
       <c r="H155" s="4" t="n">
         <v>39.46389660070852</v>
@@ -9981,10 +9981,10 @@
         <v>23</v>
       </c>
       <c r="F156" s="4" t="n">
-        <v>1.942836840412543</v>
+        <v>3.119758720222467</v>
       </c>
       <c r="G156" s="4" t="n">
-        <v>2681.114839769309</v>
+        <v>4305.267033907005</v>
       </c>
       <c r="H156" s="4" t="n">
         <v>39.45075015715322</v>
@@ -10042,10 +10042,10 @@
         <v>19</v>
       </c>
       <c r="F157" s="4" t="n">
-        <v>1.338172813739272</v>
+        <v>2.628013244678785</v>
       </c>
       <c r="G157" s="4" t="n">
-        <v>1846.678482960195</v>
+        <v>3626.658277656724</v>
       </c>
       <c r="H157" s="4" t="n">
         <v>44.52197299898833</v>
@@ -10103,10 +10103,10 @@
         <v>20</v>
       </c>
       <c r="F158" s="4" t="n">
-        <v>1.474825221819598</v>
+        <v>2.760117095103149</v>
       </c>
       <c r="G158" s="4" t="n">
-        <v>2035.258806111045</v>
+        <v>3808.961591242345</v>
       </c>
       <c r="H158" s="4" t="n">
         <v>44.50440810297314</v>
@@ -10164,10 +10164,10 @@
         <v>21</v>
       </c>
       <c r="F159" s="4" t="n">
-        <v>1.618119726992598</v>
+        <v>2.89297321376539</v>
       </c>
       <c r="G159" s="4" t="n">
-        <v>2233.005223249786</v>
+        <v>3992.303034996239</v>
       </c>
       <c r="H159" s="4" t="n">
         <v>44.48843509012828</v>
@@ -10225,10 +10225,10 @@
         <v>22</v>
       </c>
       <c r="F160" s="4" t="n">
-        <v>1.768056329258272</v>
+        <v>3.026670939759082</v>
       </c>
       <c r="G160" s="4" t="n">
-        <v>2439.917734376416</v>
+        <v>4176.805896867533</v>
       </c>
       <c r="H160" s="4" t="n">
         <v>44.47384691522967</v>
@@ -10286,10 +10286,10 @@
         <v>23</v>
       </c>
       <c r="F161" s="4" t="n">
-        <v>1.924635028616621</v>
+        <v>3.161298036570799</v>
       </c>
       <c r="G161" s="4" t="n">
-        <v>2655.996339490937</v>
+        <v>4362.591290467702</v>
       </c>
       <c r="H161" s="4" t="n">
         <v>44.46047094942217</v>
@@ -10347,10 +10347,10 @@
         <v>19</v>
       </c>
       <c r="F162" s="4" t="n">
-        <v>1.325831325928122</v>
+        <v>2.662303222373487</v>
       </c>
       <c r="G162" s="4" t="n">
-        <v>1829.647229780809</v>
+        <v>3673.978446875412</v>
       </c>
       <c r="H162" s="4" t="n">
         <v>49.53269670863701</v>
@@ -10408,10 +10408,10 @@
         <v>20</v>
       </c>
       <c r="F163" s="4" t="n">
-        <v>1.46122343787078</v>
+        <v>2.796130746791354</v>
       </c>
       <c r="G163" s="4" t="n">
-        <v>2016.488344261677</v>
+        <v>3858.660430572069</v>
       </c>
       <c r="H163" s="4" t="n">
         <v>49.5148300329157</v>
@@ -10469,10 +10469,10 @@
         <v>21</v>
       </c>
       <c r="F164" s="4" t="n">
-        <v>1.603196389227383</v>
+        <v>2.930720354945993</v>
       </c>
       <c r="G164" s="4" t="n">
-        <v>2212.411017133788</v>
+        <v>4044.394089825471</v>
       </c>
       <c r="H164" s="4" t="n">
         <v>49.49858278528747</v>
@@ -10530,10 +10530,10 @@
         <v>22</v>
       </c>
       <c r="F165" s="4" t="n">
-        <v>1.751750179997928</v>
+        <v>3.066162551615942</v>
       </c>
       <c r="G165" s="4" t="n">
-        <v>2417.415248397141</v>
+        <v>4231.30432123</v>
       </c>
       <c r="H165" s="4" t="n">
         <v>49.48374431321336</v>
@@ -10591,10 +10591,10 @@
         <v>23</v>
       </c>
       <c r="F166" s="4" t="n">
-        <v>1.906884810182418</v>
+        <v>3.202546245414422</v>
       </c>
       <c r="G166" s="4" t="n">
-        <v>2631.501038051736</v>
+        <v>4419.513818671902</v>
       </c>
       <c r="H166" s="4" t="n">
         <v>49.47013898415438</v>
@@ -10652,10 +10652,10 @@
         <v>19</v>
       </c>
       <c r="F167" s="4" t="n">
-        <v>1.313791147870646</v>
+        <v>2.696355647207897</v>
       </c>
       <c r="G167" s="4" t="n">
-        <v>1813.031784061492</v>
+        <v>3720.970793146898</v>
       </c>
       <c r="H167" s="4" t="n">
         <v>54.54336736425412</v>
@@ -10713,10 +10713,10 @@
         <v>20</v>
       </c>
       <c r="F168" s="4" t="n">
-        <v>1.447953733022461</v>
+        <v>2.831894904413269</v>
       </c>
       <c r="G168" s="4" t="n">
-        <v>1998.176151570997</v>
+        <v>3908.014968090311</v>
       </c>
       <c r="H168" s="4" t="n">
         <v>54.52519911800551</v>
@@ -10774,10 +10774,10 @@
         <v>21</v>
       </c>
       <c r="F169" s="4" t="n">
-        <v>1.58863739547764</v>
+        <v>2.96820599285485</v>
       </c>
       <c r="G169" s="4" t="n">
-        <v>2192.319605759143</v>
+        <v>4096.124270139693</v>
       </c>
       <c r="H169" s="4" t="n">
         <v>54.50867783257431</v>
@@ -10835,10 +10835,10 @@
         <v>22</v>
       </c>
       <c r="F170" s="4" t="n">
-        <v>1.735842135236181</v>
+        <v>3.105380574920552</v>
       </c>
       <c r="G170" s="4" t="n">
-        <v>2395.46214662593</v>
+        <v>4285.425193390362</v>
       </c>
       <c r="H170" s="4" t="n">
         <v>54.49358924884812</v>
@@ -10896,10 +10896,10 @@
         <v>23</v>
       </c>
       <c r="F171" s="4" t="n">
-        <v>1.889567952298086</v>
+        <v>3.243508696417081</v>
       </c>
       <c r="G171" s="4" t="n">
-        <v>2607.603774171359</v>
+        <v>4476.042001055572</v>
       </c>
       <c r="H171" s="4" t="n">
         <v>54.47975473135642</v>
@@ -10957,10 +10957,10 @@
         <v>19</v>
       </c>
       <c r="F172" s="4" t="n">
-        <v>1.30204031264108</v>
+        <v>2.730174853572195</v>
       </c>
       <c r="G172" s="4" t="n">
-        <v>1796.815631444691</v>
+        <v>3767.641297929629</v>
       </c>
       <c r="H172" s="4" t="n">
         <v>59.55398531509285</v>
@@ -11018,10 +11018,10 @@
         <v>20</v>
       </c>
       <c r="F173" s="4" t="n">
-        <v>1.435002918302513</v>
+        <v>2.867414120238351</v>
       </c>
       <c r="G173" s="4" t="n">
-        <v>1980.304027257467</v>
+        <v>3957.031485928924</v>
       </c>
       <c r="H173" s="4" t="n">
         <v>59.53551572877614</v>
@@ -11079,10 +11079,10 @@
         <v>21</v>
       </c>
       <c r="F174" s="4" t="n">
-        <v>1.574428275326359</v>
+        <v>3.005434898881416</v>
       </c>
       <c r="G174" s="4" t="n">
-        <v>2172.711019950375</v>
+        <v>4147.500160456354</v>
       </c>
       <c r="H174" s="4" t="n">
         <v>59.51872062181839</v>
@@ -11140,10 +11140,10 @@
         <v>22</v>
       </c>
       <c r="F175" s="4" t="n">
-        <v>1.720316383712617</v>
+        <v>3.144330001570435</v>
       </c>
       <c r="G175" s="4" t="n">
-        <v>2374.036609523412</v>
+        <v>4339.1754021672</v>
       </c>
       <c r="H175" s="4" t="n">
         <v>59.50338212954217</v>
@@ -11201,10 +11201,10 @@
         <v>23</v>
       </c>
       <c r="F176" s="4" t="n">
-        <v>1.87266724346129</v>
+        <v>3.284190603517176</v>
       </c>
       <c r="G176" s="4" t="n">
-        <v>2584.28079597658</v>
+        <v>4532.183032853703</v>
       </c>
       <c r="H176" s="4" t="n">
         <v>59.48931861451865</v>

</xml_diff>